<commit_message>
Finished tokenized download manager, some craftable-domain decoupling
</commit_message>
<xml_diff>
--- a/WorkBot/refactor-experimental/data/order_archive/DUTCH VALLEY FOOD DIST/DUTCH VALLEY FOOD DIST_Bakery_20251109.xlsx
+++ b/WorkBot/refactor-experimental/data/order_archive/DUTCH VALLEY FOOD DIST/DUTCH VALLEY FOOD DIST_Bakery_20251109.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,6 +551,114 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>462225</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Joe Tea - Mango Lemonade</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>22.49</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>22.49</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>462180</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Joe Tea - Kiwi Strawberry</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>22.49</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>44.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>462105</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Joe Tea - Classic Lemonade</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>22.49</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>44.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>220252</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Chocolate Block - Bronze Medal</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>325.12</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1625.60</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>